<commit_message>
Enforce single admin credentials, single active session with real-time kickout, and remove email/phone from participants
</commit_message>
<xml_diff>
--- a/apps/web/public/sample_participants.xlsx
+++ b/apps/web/public/sample_participants.xlsx
@@ -397,14 +397,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:D6"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="28.83203125" customWidth="1"/>
-    <col min="5" max="5" width="28.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -420,12 +418,6 @@
       <c r="D1" t="str">
         <v>college</v>
       </c>
-      <c r="E1" t="str">
-        <v>email</v>
-      </c>
-      <c r="F1" t="str">
-        <v>phone</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -440,12 +432,6 @@
       <c r="D2" t="str">
         <v>Black Pearl Academy</v>
       </c>
-      <c r="E2" t="str">
-        <v>jack@caribbean.edu</v>
-      </c>
-      <c r="F2" t="str">
-        <v>9876543210</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -460,12 +446,6 @@
       <c r="D3" t="str">
         <v>Port Royal Institute</v>
       </c>
-      <c r="E3" t="str">
-        <v>will@portroyal.edu</v>
-      </c>
-      <c r="F3" t="str">
-        <v>9876543211</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -480,12 +460,6 @@
       <c r="D4" t="str">
         <v>Governor High School</v>
       </c>
-      <c r="E4" t="str">
-        <v>elizabeth@portroyal.edu</v>
-      </c>
-      <c r="F4" t="str">
-        <v>9876543212</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -500,12 +474,6 @@
       <c r="D5" t="str">
         <v>Isla de Muerta College</v>
       </c>
-      <c r="E5" t="str">
-        <v>barbossa@tortuga.org</v>
-      </c>
-      <c r="F5" t="str">
-        <v>9876543213</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -520,16 +488,10 @@
       <c r="D6" t="str">
         <v>Mystic Bayou University</v>
       </c>
-      <c r="E6" t="str">
-        <v>tiadalma@calypso.net</v>
-      </c>
-      <c r="F6" t="str">
-        <v>9876543214</v>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>